<commit_message>
Presupuesto: camisetas del equipo + costo de la avanzada del jueves + pestaña de tallas
- Camisetas del equipo (~56 × est.) y Avanzada 3-sep (porción casa + 3 comidas) agregadas
  al Resumen. Meta (= costo) recalculada a ~$575,881; brecha a cubrir con recaudación
  variable = $334,631.
- Pestaña Camisetas: distribución de tallas recopiladas + a quién le falta (Paul, Frank,
  Sor, ampliados, sin-formulario). Backups excluidos (no son equipo per se).
- estado.json pendientes: flujo de caja (sesión aparte), tarifa de la avanzada, tallas.
- preparacion/MODELO_FLUJO_CAJA.md: encuadre de la sesión de tesorería (no construido aún).

https://claude.ai/code/session_016scja59CycFFrqKgYsUPWh
</commit_message>
<xml_diff>
--- a/Finanzas_ETC88.xlsx
+++ b/Finanzas_ETC88.xlsx
@@ -18,7 +18,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transporte" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recaudación" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pagos Equipo" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cómo usar" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Camisetas" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cómo usar" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +58,11 @@
       <b val="1"/>
       <color rgb="00B25028"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B25028"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -131,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -181,6 +187,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -546,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -774,178 +781,220 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Imprevistos 5%</t>
+          <t>Camisetas del equipo (~56 × est.)</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>22000</v>
+        <v>19600</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>23900</v>
+        <v>22400</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>25000</v>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
+        <v>28000</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Tallas PARCIALES (ver pestaña Camisetas); faltan invitados pendientes + Paul, Frank y la Sor. Mockup tras el Design System.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>Avanzada jueves 3-sep (porción casa + 3 comidas del equipo que adelanta)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>CONFIRMAR con la casa la tarifa de noche/día extra; depende de cuántos adelantan (cocina). Desayuno + almuerzo + cena de ese día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Imprevistos 5%</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>22000</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>23900</v>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Casa SIN exención ($2,300/p × 100) — alternativa</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B16" s="4" t="n">
         <v>230000</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C16" s="4" t="n">
         <v>230000</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D16" s="4" t="n">
         <v>230000</v>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Si NO se consigue exención: reemplaza la línea de casa (no se suma aquí)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>TOTAL ESTIMADO (con exención)</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
-        <v>477000</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>509881</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>539800</v>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="B18" s="6" t="n">
+        <v>511600</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>552281</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>591800</v>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Casa a 100 personas; precios ESTIMADOS a validar en F1</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>BRECHA Y RECAUDACIÓN</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Monto</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>(+) Costo estimado base (con exención)</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>509881</v>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Estimado · suma de arriba; precios a validar en F1</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>(+) Deuda inicial al Consejo (10% casa)</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>23600</v>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Juan Manuel pagó 5-mar; ya devuelto. Arrancamos en NEGATIVO.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>(=) Total a cubrir = META de recaudación</t>
+          <t>(+) Costo estimado base (con exención)</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>533481</v>
+        <v>552281</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>La meta NO es un número fijo: es este costo total.</t>
+          <t>Estimado · suma de arriba; precios a validar en F1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>(-) Cuotas participantes (~53 × $3,000)</t>
+          <t>(+) Deuda inicial al Consejo (10% casa)</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>159000</v>
+        <v>23600</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Para completar 100 en la casa · confirmado $3,000/participante</t>
+          <t>Juan Manuel pagó 5-mar; ya devuelto. Arrancamos en NEGATIVO.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>(-) Cuotas equipo (47 × $1,500–2,000)</t>
+          <t>(=) Total a cubrir = META de recaudación</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>82250</v>
+        <v>575881</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>[PROPUESTA] $500/mes · SIN CERRAR · rango $70,500–$94,000</t>
+          <t>La meta NO es un número fijo: es este costo total.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
+          <t>(-) Cuotas participantes (~53 × $3,000)</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>159000</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Para completar 100 en la casa · confirmado $3,000/participante</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>(-) Cuotas equipo (47 × $1,500–2,000)</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>82250</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>[PROPUESTA] $500/mes · SIN CERRAR · rango $70,500–$94,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>(=) BRECHA: rifa + venta de comida + donaciones</t>
         </is>
       </c>
-      <c r="B26" s="4" t="n">
-        <v>292231</v>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="B28" s="4" t="n">
+        <v>334631</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Montos VARIABLES (lo que se recaude). Rifa = primera actividad. Donaciones = responsabilidad de Directores.</t>
         </is>
@@ -978,7 +1027,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>RECAUDACIÓN · la META = costo total $533,481 (cuotas + rifa/comida + donaciones)</t>
+          <t>RECAUDACIÓN · la META = costo total $575,881 (cuotas + rifa/comida + donaciones)</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1208,7 @@
         <v/>
       </c>
       <c r="B10" s="4" t="n">
-        <v>292231</v>
+        <v>334631</v>
       </c>
       <c r="C10" s="3" t="inlineStr"/>
       <c r="D10" s="3" t="inlineStr"/>
@@ -2791,6 +2840,348 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>CAMISETAS DEL EQUIPO · tallas (parcial) — mockup tras el Design System</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>CON talla</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>de 52 del equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>FALTAN talla</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>pedir antes de imprimir</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>A QUIÉNES FALTA LA TALLA:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Área</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Motivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Frank Morales</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>asesores</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Johanny García</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>asesores_cocina</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Mary "Peta" Morales</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>asesores_cocina</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Leticia González</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>asesores_diocesanos</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Marleny</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>asesores_diocesanos</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Sandrita</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>asesores_diocesanos</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Padre Paul Ramírez</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>asesores_espirituales</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Sor Angelina Lebrón</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>asesores_espirituales</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Olanlly</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>cocina</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Pamela</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>cocina</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Daylin</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>musica</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>sin formulario</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2798,163 +3189,163 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>FINANZAS ETC 88 — HOJA VIVA · v8 · 2-jun-2026</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr"/>
+      <c r="A2" s="19" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Cómo se usa:</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="19" t="inlineStr">
         <is>
           <t>1. La pestaña Resumen es la foto ejecutiva. Lee primero.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>2. Las pestañas por área (Casa, Cocina-Compras, Materiales, Guías, Música, Formaciones, Transporte)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">   son lo que cada coordinador entrega y refina en F1 (14-jun). Precios son ESTIMADOS a validar.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>3. Menú es estructura sin precios; cocina lo refina y de ahí salen las cantidades de Cocina-Compras.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>4. Recaudación: la META = el costo total. Se cubre con cuotas (participantes + equipo) +</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">   rifa + venta de comida + donaciones (montos VARIABLES, lo que se recaude).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>5. Pagos Equipo: cuota PROPUESTA de $500/mes (total $1,500–2,000/persona). SIN CERRAR — la decide la Dirección.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr"/>
+      <c r="A11" s="19" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>CONTEXTO CRÍTICO:</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>• Arrancamos en NEGATIVO: $23,600 (10% reserva casa pagada por Juan Manuel ya devuelto al Consejo).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t xml:space="preserve">  Es la PRIMERA deuda a cubrir con la recaudación.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>• La casa INCLUYE gas y limpieza (no se compra). Con exención: $2,000/p; sin exención: $2,300/p.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>• Casa tiene sonido (música solo lleva respaldo).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>• Piso de personas: completar 100 en la casa (≈47 operativos + ~53 participantes).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr"/>
+      <c r="A18" s="19" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>PENDIENTES PARA CERRAR EL PRESUPUESTO:</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>• Cerrar el monto final de la cuota del equipo (propuesta $500/mes, total $1,500–2,000).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>• Gestionar exención con el Padre Paul (impacto ~$30,000 a 100 personas).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>• Cotizar transporte (3 empresas) · fijar fecha límite (también biblias y peces).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>• Banderín: diseño + cotización.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>• Confirmar el conteo final para completar 100 en la casa (afecta peces, biblias, comida).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>• Donaciones en especie: arroz, habichuelas, aceite (el ETC 79 los consiguió donados).</t>
         </is>

</xml_diff>

<commit_message>
Petra (no Peta) + convivencia/ensayo-con-almuerzo/bizcocho post-ETC al presupuesto
- Corrección de nombre: Mary "Petra" Morales (era "Peta") en fuentes y docs.
- Resumen + pestaña Formaciones: agregadas Convivencia (22-ago, ~12K), Ensayo General
  con almuerzo del equipo (23-ago, ~16K) y Bienvenida post-ETC / bizcocho (9-sep, ~3K).
  Estaban en el detalle pero no en el total.
- Meta (= costo) recalculada a ~$606,881; brecha a cubrir con recaudación variable = $365,631.
- TODO PASS.

https://claude.ai/code/session_016scja59CycFFrqKgYsUPWh
</commit_message>
<xml_diff>
--- a/Finanzas_ETC88.xlsx
+++ b/Finanzas_ETC88.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -764,7 +764,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Formaciones (5 sesiones · refrigerio + local)</t>
+          <t>Formaciones F1–F5 (5 sesiones · refrigerio + local)</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
@@ -781,220 +781,283 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Camisetas del equipo (~56 × est.)</t>
+          <t>Convivencia del equipo (22-ago · día completo)</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>19600</v>
+        <v>8000</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>22400</v>
+        <v>12000</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>28000</v>
+        <v>18000</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Tallas PARCIALES (ver pestaña Camisetas); faltan invitados pendientes + Paul, Frank y la Sor. Mockup tras el Design System.</t>
+          <t>Miniretiro; confirmar si incluye almuerzo del equipo y local</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Avanzada jueves 3-sep (porción casa + 3 comidas del equipo que adelanta)</t>
+          <t>Ensayo General (23-ago · INCLUYE el almuerzo del equipo)</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>15000</v>
+        <v>12000</v>
       </c>
       <c r="C14" s="4" t="n">
+        <v>16000</v>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>20000</v>
       </c>
-      <c r="D14" s="4" t="n">
-        <v>24000</v>
-      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>CONFIRMAR con la casa la tarifa de noche/día extra; depende de cuántos adelantan (cocina). Desayuno + almuerzo + cena de ese día.</t>
+          <t>Almuerzo ~52 personas + refrigerio + local</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Imprevistos 5%</t>
+          <t>Bienvenida post-ETC (9-sep · bizcocho)</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>22000</v>
+        <v>2000</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>23900</v>
+        <v>3000</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>25000</v>
-      </c>
-      <c r="E15" s="3" t="inlineStr"/>
+        <v>4500</v>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Bizcocho de bienvenida de los nuevos (1ra reunión post-retiro)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>Camisetas del equipo (~56 × est.)</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>22400</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>28000</v>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Tallas PARCIALES (ver pestaña Camisetas); faltan invitados pendientes + Paul, Frank y la Sor. Mockup tras el Design System.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Avanzada jueves 3-sep (porción casa + 3 comidas del equipo que adelanta)</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>15000</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>24000</v>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>CONFIRMAR con la casa la tarifa de noche/día extra; depende de cuántos adelantan (cocina). Desayuno + almuerzo + cena de ese día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Imprevistos 5%</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>22000</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>23900</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
           <t>Casa SIN exención ($2,300/p × 100) — alternativa</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B19" s="4" t="n">
         <v>230000</v>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C19" s="4" t="n">
         <v>230000</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D19" s="4" t="n">
         <v>230000</v>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Si NO se consigue exención: reemplaza la línea de casa (no se suma aquí)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr"/>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>TOTAL ESTIMADO (con exención)</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n">
-        <v>511600</v>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>552281</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>591800</v>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="B21" s="6" t="n">
+        <v>533600</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>583281</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>634300</v>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>Casa a 100 personas; precios ESTIMADOS a validar en F1</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>BRECHA Y RECAUDACIÓN</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Monto</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>(+) Costo estimado base (con exención)</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>552281</v>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>Estimado · suma de arriba; precios a validar en F1</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>(+) Deuda inicial al Consejo (10% casa)</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="n">
-        <v>23600</v>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Juan Manuel pagó 5-mar; ya devuelto. Arrancamos en NEGATIVO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>(=) Total a cubrir = META de recaudación</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="n">
-        <v>575881</v>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>La meta NO es un número fijo: es este costo total.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>(-) Cuotas participantes (~53 × $3,000)</t>
+          <t>(+) Costo estimado base (con exención)</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>159000</v>
+        <v>583281</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Para completar 100 en la casa · confirmado $3,000/participante</t>
+          <t>Estimado · suma de arriba; precios a validar en F1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>(-) Cuotas equipo (47 × $1,500–2,000)</t>
+          <t>(+) Deuda inicial al Consejo (10% casa)</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>82250</v>
+        <v>23600</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>[PROPUESTA] $500/mes · SIN CERRAR · rango $70,500–$94,000</t>
+          <t>Juan Manuel pagó 5-mar; ya devuelto. Arrancamos en NEGATIVO.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
+          <t>(=) Total a cubrir = META de recaudación</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>606881</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>La meta NO es un número fijo: es este costo total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>(-) Cuotas participantes (~53 × $3,000)</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>159000</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Para completar 100 en la casa · confirmado $3,000/participante</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>(-) Cuotas equipo (47 × $1,500–2,000)</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>82250</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>[PROPUESTA] $500/mes · SIN CERRAR · rango $70,500–$94,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
           <t>(=) BRECHA: rifa + venta de comida + donaciones</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n">
-        <v>334631</v>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="B31" s="4" t="n">
+        <v>365631</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>Montos VARIABLES (lo que se recaude). Rifa = primera actividad. Donaciones = responsabilidad de Directores.</t>
         </is>
@@ -1027,7 +1090,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>RECAUDACIÓN · la META = costo total $575,881 (cuotas + rifa/comida + donaciones)</t>
+          <t>RECAUDACIÓN · la META = costo total $606,881 (cuotas + rifa/comida + donaciones)</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1271,7 @@
         <v/>
       </c>
       <c r="B10" s="4" t="n">
-        <v>334631</v>
+        <v>365631</v>
       </c>
       <c r="C10" s="3" t="inlineStr"/>
       <c r="D10" s="3" t="inlineStr"/>
@@ -3018,7 +3081,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Mary "Peta" Morales</t>
+          <t>Mary "Petra" Morales</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -5686,7 +5749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5883,7 +5946,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Convivencia (miniretiro)</t>
+          <t>Convivencia (miniretiro · día completo)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -5892,22 +5955,22 @@
         </is>
       </c>
       <c r="C10" s="4" t="n">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>2000</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>1500</v>
+        <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>6500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Ensayo General</t>
+          <t>Ensayo General (incluye almuerzo del equipo)</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -5916,7 +5979,7 @@
         </is>
       </c>
       <c r="C11" s="4" t="n">
-        <v>2000</v>
+        <v>15000</v>
       </c>
       <c r="D11" s="14" t="n">
         <v>0</v>
@@ -5925,7 +5988,7 @@
         <v>1000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>3000</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="12">
@@ -5952,18 +6015,42 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Bienvenida post-ETC (bizcocho)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>9-sep</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>TOTAL FORMACIONES</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr"/>
-      <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr"/>
-      <c r="E14" s="5" t="inlineStr"/>
-      <c r="F14" s="6" t="n">
-        <v>26100</v>
+      <c r="B15" s="5" t="inlineStr"/>
+      <c r="C15" s="5" t="inlineStr"/>
+      <c r="D15" s="5" t="inlineStr"/>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="6" t="n">
+        <v>47600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>